<commit_message>
Update card balance numbers and translations
Adjust multiple card balance values and related metadata, and regenerate artifacts. Notable changes: BlazeInferno BaseBurning 7/9 → 4/7; Lihuo and Kunai burning values increased to 6/9; KujiProtection Resist 3 → 2 and its Chinese description fixed; IaiStrike cost 1 → 2; StoneSummon BaseBlock 2 → 3 (Upgrade 3 → 4); several cards had damage/upgradeDamage and Dex adjustments (e.g. MusashiThrust cost 3 → 2 and add UpgradeDamage 21, MusashiVoidSlash damage lowered, MusashiAdvancingFountain Dex reduced, several other Attack/Block values tweaked). Also added many balance translation stub files, updated balance CSV/Excel, regenerated CardBalance.g.cs and added a UID file, and updated distribution binaries and generated markdown.
</commit_message>
<xml_diff>
--- a/balance/NinjaMod_Balance.xlsx
+++ b/balance/NinjaMod_Balance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--UnityProject\RunminG-Lab\SlaytheSpire2_mod\balance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC56AA50-AC4B-41D3-95A4-A95F7B252B16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12961CEC-CBD8-4294-91B7-A68F1E6F9745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{E1875C0B-A6BC-4540-87E7-A85DB8E4E18A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{E1875C0B-A6BC-4540-87E7-A85DB8E4E18A}"/>
   </bookViews>
   <sheets>
     <sheet name="说明" sheetId="5" r:id="rId1"/>
@@ -8052,7 +8052,7 @@
         <v>6</v>
       </c>
       <c r="BA19" s="12">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="BB19" s="12"/>
       <c r="BC19" s="12"/>
@@ -8162,7 +8162,9 @@
       <c r="AZ20" s="12">
         <v>9</v>
       </c>
-      <c r="BA20" s="12"/>
+      <c r="BA20" s="12">
+        <v>11</v>
+      </c>
       <c r="BB20" s="12"/>
       <c r="BC20" s="12"/>
       <c r="BD20" s="12"/>

</xml_diff>

<commit_message>
Add ninja cards, images and balance updates
Add many new ninja cards and portraits, plus supporting C# card and power classes, scripts and balance data. Updated NinjaMod/balance/cards.json with numerous new card entries (e.g. NinjaToolPrep, HandSwap, FireSpread, EmberRecovery, FanWind, MusashiDreamStrike, MusashiCrimson, BladeFlow, Wildfire, StoneHide, MusashiPeerless, BloodFireTransfer, ShadowBreath, NimbleStep, CovertOps, FlameDance, Earthquake) and applied targeted tweaks to existing cards. Notable gameplay changes: KusariGama now deals 8(11) and applies 2 Weak when target has Bleed; SwallowReturn cost reduced to 0 and now draws 1(2) cards if the target has Bleed; Susanoo/SoulChase text clarified for per-hit bleed sequencing. Also added/imported portrait images and import metadata, updated generated balance code/file and distribution artifacts, and added helper scripts for balance application.
</commit_message>
<xml_diff>
--- a/balance/NinjaMod_Balance.xlsx
+++ b/balance/NinjaMod_Balance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--UnityProject\RunminG-Lab\SlaytheSpire2_mod\balance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1372737D-D536-494B-9A28-FEDF5096B330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D320F2E-0DBD-45BE-A2B6-A6BFA0FDC0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{E1875C0B-A6BC-4540-87E7-A85DB8E4E18A}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2082" uniqueCount="691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2082" uniqueCount="696">
   <si>
     <t>用途</t>
   </si>
@@ -2129,6 +2129,26 @@
   </si>
   <si>
     <t>造成 7(11) 点伤害，附加 2 层【流血】。【武藏】牌。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>追魂</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>对目标打出消耗牌堆中的所有【飞刀】（每张造成其伤害+流血）；若成功击杀，抽 2(3) 张牌。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>锁镰</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>造成 9(12) 点伤害；若目标有【流血】，额外造成 4(6) 点伤害。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>获得 3(4) 层【淬火】：本回合攻击牌每次造成伤害额外附加等同于淬火层数的【燃烧】。</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -2287,7 +2307,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2344,6 +2364,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2837,7 +2860,7 @@
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4" t="s">
-        <v>33</v>
+        <v>695</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -4202,8 +4225,8 @@
       <c r="E47" s="4">
         <v>1</v>
       </c>
-      <c r="F47" s="4" t="s">
-        <v>177</v>
+      <c r="F47" s="18" t="s">
+        <v>693</v>
       </c>
       <c r="G47" s="4" t="s">
         <v>178</v>
@@ -4212,8 +4235,8 @@
         <v>178</v>
       </c>
       <c r="I47" s="4"/>
-      <c r="J47" s="4" t="s">
-        <v>179</v>
+      <c r="J47" s="19" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
@@ -4262,8 +4285,8 @@
       <c r="E49" s="4">
         <v>3</v>
       </c>
-      <c r="F49" s="4" t="s">
-        <v>183</v>
+      <c r="F49" s="18" t="s">
+        <v>691</v>
       </c>
       <c r="G49" s="4" t="s">
         <v>184</v>
@@ -4275,7 +4298,7 @@
         <v>45</v>
       </c>
       <c r="J49" s="18" t="s">
-        <v>185</v>
+        <v>692</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="29" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Fix Bleed trigger and card balance updates
Updates gameplay and balance data to match intended behavior: Bleed now triggers on any unblocked damage source (with re-entrancy protection), Blade Flow now auto-plays Infused Shuriken in addition to Kunai/Shuriken, Bone Art gains proper upgrade scaling (11->15 Block, 2->3 Vigor), Musashi Crimson upgrade now grants 3 Quenching, and Musashi Seven Star is reclassified as an Attack. Synced related balance sources/generated files and card docs to keep data and text consistent.
</commit_message>
<xml_diff>
--- a/balance/NinjaMod_Balance.xlsx
+++ b/balance/NinjaMod_Balance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\__RunminG-Lab\SlaytheSpire2_mod\balance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD61040E-FFD2-4305-8D54-1330CE58B304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{82CB2CE6-1CDB-4EB7-84A5-47F03720FC83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="28800" windowHeight="15370" xr2:uid="{F9B761CB-8BAA-4208-8885-F2E68FD70C6F}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="28800" windowHeight="15370" xr2:uid="{5A12750B-E6DB-4A4C-98D0-2B3CA8B56BA9}"/>
   </bookViews>
   <sheets>
     <sheet name="说明" sheetId="5" r:id="rId1"/>
@@ -464,7 +464,7 @@
     <t>MusashiCrimson</t>
   </si>
   <si>
-    <t>获得 2 层【淬火】。</t>
+    <t>获得 2(3) 层【淬火】。</t>
   </si>
   <si>
     <t>武藏：迅光三角剑</t>
@@ -668,7 +668,7 @@
     <t>BoneArt</t>
   </si>
   <si>
-    <t>获得 11 点格挡，并获得 2 点【活力】。</t>
+    <t>获得 11(15) 点格挡，并获得 2(3) 点【活力】。</t>
   </si>
   <si>
     <t>九字护身法</t>
@@ -1727,7 +1727,7 @@
     <t>常量变量，保持 JSON 格式。</t>
   </si>
   <si>
-    <t>{"Vigor": 2}</t>
+    <t>{"Vigor": 2, "VigorUpgraded": 3}</t>
   </si>
   <si>
     <t>{"Count": 2}</t>
@@ -2905,7 +2905,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7826F2A5-C417-4819-A760-8F02386D98B3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEC746EB-6BED-40CF-8672-F25B09236A0D}">
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3004,7 +3004,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AFC82F3-802E-4747-A3CF-11B47B8E7849}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82F4D94A-EA2D-49D3-9C90-B48D4E863FA5}">
   <dimension ref="A1:J78"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4261,7 +4261,7 @@
         <v>78</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E41" s="9">
         <v>2</v>
@@ -5409,93 +5409,93 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J78" xr:uid="{9AFC82F3-802E-4747-A3CF-11B47B8E7849}"/>
+  <autoFilter ref="A1:J78" xr:uid="{82F4D94A-EA2D-49D3-9C90-B48D4E863FA5}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="A8" location="'卡牌数值'!D$1" display="打开" xr:uid="{16D74CA3-8BD6-4124-AEEC-B2D89C9724A2}"/>
-    <hyperlink ref="A7" location="'卡牌数值'!E$1" display="打开" xr:uid="{D9C60434-E0B3-47B4-9D67-6D246B1243E9}"/>
-    <hyperlink ref="A57" location="'卡牌数值'!F$1" display="打开" xr:uid="{181DDF4A-7237-4D5C-AED5-3ABA3D8ED95C}"/>
-    <hyperlink ref="A25" location="'卡牌数值'!G$1" display="打开" xr:uid="{C3A4FFC7-1E49-4824-9B94-2A2DC1F1555F}"/>
-    <hyperlink ref="A6" location="'卡牌数值'!H$1" display="打开" xr:uid="{2FE3C26B-AD59-4DC5-A790-1790396C8A30}"/>
-    <hyperlink ref="A10" location="'卡牌数值'!I$1" display="打开" xr:uid="{A4D61A3F-3F94-4390-BFCD-122A802AEBFB}"/>
-    <hyperlink ref="A26" location="'卡牌数值'!J$1" display="打开" xr:uid="{CEB3C2E8-C072-476A-8442-53FE9DF8290E}"/>
-    <hyperlink ref="A28" location="'卡牌数值'!K$1" display="打开" xr:uid="{A8B969B4-AF29-4DCE-A053-61745F74AF91}"/>
-    <hyperlink ref="A11" location="'卡牌数值'!L$1" display="打开" xr:uid="{2514AAF7-904A-41CB-9232-9A8514311331}"/>
-    <hyperlink ref="A9" location="'卡牌数值'!M$1" display="打开" xr:uid="{FB807F28-2B40-4D24-BF6C-C64A18CCD4B3}"/>
-    <hyperlink ref="A58" location="'卡牌数值'!N$1" display="打开" xr:uid="{55811AA8-905A-4C5C-AF95-04B1E56EC22B}"/>
-    <hyperlink ref="A61" location="'卡牌数值'!O$1" display="打开" xr:uid="{CD43B91F-539A-429B-A0F4-0DD1AB5D5FBC}"/>
-    <hyperlink ref="A62" location="'卡牌数值'!P$1" display="打开" xr:uid="{065C7AFD-A424-4C3A-9512-E56E8D561D8E}"/>
-    <hyperlink ref="A12" location="'卡牌数值'!Q$1" display="打开" xr:uid="{CE97B9BD-C9D1-49E6-84D6-00D1F06B9E90}"/>
-    <hyperlink ref="A32" location="'卡牌数值'!R$1" display="打开" xr:uid="{992F7379-A952-45BB-8759-A0C76D897C69}"/>
-    <hyperlink ref="A37" location="'卡牌数值'!S$1" display="打开" xr:uid="{9DF8DF79-259F-43DE-A120-81B93510C59A}"/>
-    <hyperlink ref="A34" location="'卡牌数值'!T$1" display="打开" xr:uid="{CA5EB6FC-7963-442F-B773-A52EF1FACD5D}"/>
-    <hyperlink ref="A36" location="'卡牌数值'!U$1" display="打开" xr:uid="{229F83EE-EE49-43E4-AA53-6E173867CA32}"/>
-    <hyperlink ref="A27" location="'卡牌数值'!V$1" display="打开" xr:uid="{F0B10ADA-3C73-462A-91EE-0731B070D3EF}"/>
-    <hyperlink ref="A24" location="'卡牌数值'!W$1" display="打开" xr:uid="{748C3290-3F4A-433D-8916-440A34A91E85}"/>
-    <hyperlink ref="A59" location="'卡牌数值'!X$1" display="打开" xr:uid="{9E9FA501-15B7-414A-A9F7-949740586E90}"/>
-    <hyperlink ref="A63" location="'卡牌数值'!Y$1" display="打开" xr:uid="{F4960A40-7990-4AA2-9FCE-62CD450F732A}"/>
-    <hyperlink ref="A60" location="'卡牌数值'!Z$1" display="打开" xr:uid="{4988C555-3513-406C-988F-6282B2C20C19}"/>
-    <hyperlink ref="A55" location="'卡牌数值'!AA$1" display="打开" xr:uid="{D522253C-47C7-4DD5-A6C4-919EC705712A}"/>
-    <hyperlink ref="A76" location="'卡牌数值'!AB$1" display="打开" xr:uid="{E978E76E-6E4F-4743-AF8C-4C885E69291A}"/>
-    <hyperlink ref="A78" location="'卡牌数值'!AC$1" display="打开" xr:uid="{6B079010-2F2D-41C2-92BA-296ADBE7C057}"/>
-    <hyperlink ref="A77" location="'卡牌数值'!AD$1" display="打开" xr:uid="{C22BF1E1-3E0D-441F-BBAC-797334FA9A49}"/>
-    <hyperlink ref="A67" location="'卡牌数值'!AE$1" display="打开" xr:uid="{0CB32956-8A95-4087-BDE3-3996580685BE}"/>
-    <hyperlink ref="A65" location="'卡牌数值'!AF$1" display="打开" xr:uid="{0653DC4B-1889-4812-8BFA-27EF259C30B5}"/>
-    <hyperlink ref="A66" location="'卡牌数值'!AG$1" display="打开" xr:uid="{B86134C2-BA49-4B11-A97E-0CD15104FC3E}"/>
-    <hyperlink ref="A17" location="'卡牌数值'!AH$1" display="打开" xr:uid="{CE609D39-D076-457D-96CE-C7789FC1A080}"/>
-    <hyperlink ref="A70" location="'卡牌数值'!AI$1" display="打开" xr:uid="{10FD33C8-93A0-4304-94C8-0654719120F7}"/>
-    <hyperlink ref="A38" location="'卡牌数值'!AJ$1" display="打开" xr:uid="{891AFAB3-5907-446B-8D39-98C3570F2D61}"/>
-    <hyperlink ref="A41" location="'卡牌数值'!AK$1" display="打开" xr:uid="{1A69FCB4-E4B7-4ED3-AF80-9A011C8B4F97}"/>
-    <hyperlink ref="A39" location="'卡牌数值'!AL$1" display="打开" xr:uid="{0FB2112B-7526-43B1-899F-511A75320426}"/>
-    <hyperlink ref="A40" location="'卡牌数值'!AM$1" display="打开" xr:uid="{CCDAE4F1-5587-49FD-969D-69C34161EE56}"/>
-    <hyperlink ref="A68" location="'卡牌数值'!AN$1" display="打开" xr:uid="{EE1E3F19-EBAD-4711-840C-27EC6549A121}"/>
-    <hyperlink ref="A73" location="'卡牌数值'!AO$1" display="打开" xr:uid="{A04A6C22-EBFE-4D6B-A865-3F5BAC22EB60}"/>
-    <hyperlink ref="A75" location="'卡牌数值'!AP$1" display="打开" xr:uid="{048BD626-B4FA-4F7D-B261-DD66C8D78C44}"/>
-    <hyperlink ref="A72" location="'卡牌数值'!AQ$1" display="打开" xr:uid="{4216D299-AD93-4124-9964-304957FCDB6D}"/>
-    <hyperlink ref="A71" location="'卡牌数值'!AR$1" display="打开" xr:uid="{2FE198F4-811C-4E18-8255-B9C873CF1D25}"/>
-    <hyperlink ref="A5" location="'卡牌数值'!AS$1" display="打开" xr:uid="{56425AA4-0AAD-4F0E-8F11-7908379303B1}"/>
-    <hyperlink ref="A22" location="'卡牌数值'!AT$1" display="打开" xr:uid="{F0A120E9-9230-49E8-A4A1-7EB2C9DA9DAF}"/>
-    <hyperlink ref="A23" location="'卡牌数值'!AU$1" display="打开" xr:uid="{E57953F7-555E-433D-89DC-C68EA340144C}"/>
-    <hyperlink ref="A3" location="'卡牌数值'!AV$1" display="打开" xr:uid="{C3DE20FA-355D-40F3-93B8-1E5A8D446D5E}"/>
-    <hyperlink ref="A48" location="'卡牌数值'!AW$1" display="打开" xr:uid="{1CE0DB34-3C9D-412F-B652-E69C5A7854B8}"/>
-    <hyperlink ref="A53" location="'卡牌数值'!AX$1" display="打开" xr:uid="{DBA1DDCA-8E02-4F46-B434-028F0E52B1C5}"/>
-    <hyperlink ref="A50" location="'卡牌数值'!AY$1" display="打开" xr:uid="{2128C8FD-4A29-4C72-A65D-8D9AF0FC040B}"/>
-    <hyperlink ref="A49" location="'卡牌数值'!AZ$1" display="打开" xr:uid="{13087FB2-16CF-4C37-8E6F-D7BEE993B3ED}"/>
-    <hyperlink ref="A31" location="'卡牌数值'!BA$1" display="打开" xr:uid="{D7CE26A5-3C5B-462A-B736-C4C08D79FBBF}"/>
-    <hyperlink ref="A51" location="'卡牌数值'!BB$1" display="打开" xr:uid="{A40C4579-95D4-47CF-8B43-9CE1A2EC45AF}"/>
-    <hyperlink ref="A2" location="'卡牌数值'!BC$1" display="打开" xr:uid="{D09A3A57-E0D8-4372-B73D-8AC3DFD6D268}"/>
-    <hyperlink ref="A21" location="'卡牌数值'!BD$1" display="打开" xr:uid="{87F7D405-3F8D-47BA-93E9-7875D1DF644D}"/>
-    <hyperlink ref="A20" location="'卡牌数值'!BE$1" display="打开" xr:uid="{07239B15-878C-4D94-9983-BC2893F0C41C}"/>
-    <hyperlink ref="A19" location="'卡牌数值'!BF$1" display="打开" xr:uid="{487BFC69-9EC7-45C4-AB51-63AAC245F480}"/>
-    <hyperlink ref="A54" location="'卡牌数值'!BG$1" display="打开" xr:uid="{9F017C27-92C0-45FC-800C-6A4846143D7C}"/>
-    <hyperlink ref="A43" location="'卡牌数值'!BH$1" display="打开" xr:uid="{7FD1B1F0-11D3-4A79-8DE1-913318CAAA98}"/>
-    <hyperlink ref="A45" location="'卡牌数值'!BI$1" display="打开" xr:uid="{E4266A66-6F1A-421C-BCD1-E4CA60C1D84C}"/>
-    <hyperlink ref="A44" location="'卡牌数值'!BJ$1" display="打开" xr:uid="{1C2E34BA-6512-4719-9C80-31F198005E3E}"/>
-    <hyperlink ref="A46" location="'卡牌数值'!BK$1" display="打开" xr:uid="{E60D8A20-A397-44C2-953F-B7EADBD57AFE}"/>
-    <hyperlink ref="A52" location="'卡牌数值'!BL$1" display="打开" xr:uid="{4D738EAB-1603-4620-8B0C-C1B37508A2A4}"/>
-    <hyperlink ref="A47" location="'卡牌数值'!BM$1" display="打开" xr:uid="{838CE5BC-D018-49CE-BE0F-3DD8EB058170}"/>
-    <hyperlink ref="A4" location="'卡牌数值'!BN$1" display="打开" xr:uid="{CD335897-01E3-4732-A8BE-67CD55B30244}"/>
-    <hyperlink ref="A15" location="'卡牌数值'!BO$1" display="打开" xr:uid="{3203C171-FB88-40F2-8435-C2BB62558702}"/>
-    <hyperlink ref="A14" location="'卡牌数值'!BP$1" display="打开" xr:uid="{C855F57C-3BC5-4CF5-A5AE-CEEC76175F52}"/>
-    <hyperlink ref="A33" location="'卡牌数值'!BQ$1" display="打开" xr:uid="{BCE6EAEA-DAAC-4D8D-9D5B-81D6D3748748}"/>
-    <hyperlink ref="A35" location="'卡牌数值'!BR$1" display="打开" xr:uid="{921787FE-34DE-4AF9-83ED-702BA9E2CF53}"/>
-    <hyperlink ref="A56" location="'卡牌数值'!BS$1" display="打开" xr:uid="{475E4CFE-A743-4749-AE69-80D0F60BA7AE}"/>
-    <hyperlink ref="A13" location="'卡牌数值'!BT$1" display="打开" xr:uid="{2EC3609E-42EC-4D05-8496-E1B6BAB53DB2}"/>
-    <hyperlink ref="A30" location="'卡牌数值'!BU$1" display="打开" xr:uid="{800375FC-98A4-463D-97E0-EF79059D7097}"/>
-    <hyperlink ref="A42" location="'卡牌数值'!BV$1" display="打开" xr:uid="{F48A7DFB-DC74-43AB-9B29-79627B1BA1F8}"/>
-    <hyperlink ref="A18" location="'卡牌数值'!BW$1" display="打开" xr:uid="{A28BC9AF-2A8C-4A23-B65F-F03E6CF936C7}"/>
-    <hyperlink ref="A74" location="'卡牌数值'!BX$1" display="打开" xr:uid="{A10FE843-E334-46B9-92F6-F0551D29907B}"/>
-    <hyperlink ref="A69" location="'卡牌数值'!BY$1" display="打开" xr:uid="{72B43B24-324F-46F3-994B-EF2CC511B08D}"/>
-    <hyperlink ref="A64" location="'卡牌数值'!BZ$1" display="打开" xr:uid="{01DD12FF-43E3-4277-AE03-630B5C42B9B8}"/>
-    <hyperlink ref="A16" location="'卡牌数值'!CA$1" display="打开" xr:uid="{83DEA829-00B0-4AD8-A0E0-E8F64B8F43B6}"/>
-    <hyperlink ref="A29" location="'卡牌数值'!CB$1" display="打开" xr:uid="{B2F36BF5-FDFE-4921-93DD-08195170C203}"/>
+    <hyperlink ref="A8" location="'卡牌数值'!D$1" display="打开" xr:uid="{A26CD4CB-31B4-4348-9862-F81E8BB1F432}"/>
+    <hyperlink ref="A7" location="'卡牌数值'!E$1" display="打开" xr:uid="{E614DDDC-AAB6-4586-BBDA-76C4222DF317}"/>
+    <hyperlink ref="A57" location="'卡牌数值'!F$1" display="打开" xr:uid="{9B10917D-D84A-43D5-8B18-663A7F00CC3E}"/>
+    <hyperlink ref="A25" location="'卡牌数值'!G$1" display="打开" xr:uid="{4B12EDA5-93B2-4D7F-9B0B-5C2E13FE77A1}"/>
+    <hyperlink ref="A6" location="'卡牌数值'!H$1" display="打开" xr:uid="{FF334929-3AB3-4120-AC34-7FFCEFA683A1}"/>
+    <hyperlink ref="A10" location="'卡牌数值'!I$1" display="打开" xr:uid="{BFE3CB6C-1043-460C-95EE-0A2B8A1AC96A}"/>
+    <hyperlink ref="A26" location="'卡牌数值'!J$1" display="打开" xr:uid="{9F3DA9CB-481A-4321-8DDA-F7DC7102F876}"/>
+    <hyperlink ref="A28" location="'卡牌数值'!K$1" display="打开" xr:uid="{03939E20-8412-4D1A-A36D-C3C8DAE405D5}"/>
+    <hyperlink ref="A11" location="'卡牌数值'!L$1" display="打开" xr:uid="{5C481514-173F-4B4D-8CCE-02F205B21B81}"/>
+    <hyperlink ref="A9" location="'卡牌数值'!M$1" display="打开" xr:uid="{357F9C15-F97E-4260-86C7-BF038CAEF5A4}"/>
+    <hyperlink ref="A58" location="'卡牌数值'!N$1" display="打开" xr:uid="{7F053C80-B4CF-48A2-AD27-3627930B9899}"/>
+    <hyperlink ref="A61" location="'卡牌数值'!O$1" display="打开" xr:uid="{2075C932-6166-407A-AF16-68BF37EBDFF9}"/>
+    <hyperlink ref="A62" location="'卡牌数值'!P$1" display="打开" xr:uid="{CB45D135-35B9-440A-B2A2-73C562AD780A}"/>
+    <hyperlink ref="A12" location="'卡牌数值'!Q$1" display="打开" xr:uid="{75FF8EE8-B92C-442D-B1E6-5EF85D5572F6}"/>
+    <hyperlink ref="A32" location="'卡牌数值'!R$1" display="打开" xr:uid="{19FE2B8F-76B5-4783-94B6-F1520ED4B5D0}"/>
+    <hyperlink ref="A37" location="'卡牌数值'!S$1" display="打开" xr:uid="{B4E2B47A-10AB-41B8-8283-F6AFCC250049}"/>
+    <hyperlink ref="A34" location="'卡牌数值'!T$1" display="打开" xr:uid="{E2D8224B-EE87-4270-AE35-306785DE8932}"/>
+    <hyperlink ref="A36" location="'卡牌数值'!U$1" display="打开" xr:uid="{27FA45C3-16F5-4EC0-977B-1C5871FBF7F7}"/>
+    <hyperlink ref="A27" location="'卡牌数值'!V$1" display="打开" xr:uid="{916244A8-DC41-4BD3-B929-4934CE4B7608}"/>
+    <hyperlink ref="A24" location="'卡牌数值'!W$1" display="打开" xr:uid="{24078FE3-3702-4CEF-B2B9-3E434CF5280F}"/>
+    <hyperlink ref="A59" location="'卡牌数值'!X$1" display="打开" xr:uid="{5551E71A-9DB7-4904-9CD3-EABE84D8775D}"/>
+    <hyperlink ref="A63" location="'卡牌数值'!Y$1" display="打开" xr:uid="{938A46A7-C6FA-4FF3-B918-B9D6D3C0D2D3}"/>
+    <hyperlink ref="A60" location="'卡牌数值'!Z$1" display="打开" xr:uid="{AFF940A6-AEB8-4972-89D9-34A893B18326}"/>
+    <hyperlink ref="A55" location="'卡牌数值'!AA$1" display="打开" xr:uid="{C14FA6A4-8257-4E50-84BE-BE8F1F6A6E0E}"/>
+    <hyperlink ref="A76" location="'卡牌数值'!AB$1" display="打开" xr:uid="{0B2AC667-F74B-42A2-A345-5EF1022C4198}"/>
+    <hyperlink ref="A78" location="'卡牌数值'!AC$1" display="打开" xr:uid="{804F9EE2-3303-42C4-BD70-5EE55C56EF61}"/>
+    <hyperlink ref="A77" location="'卡牌数值'!AD$1" display="打开" xr:uid="{95F81A51-18F3-4506-AFCC-9A966B8CADC3}"/>
+    <hyperlink ref="A67" location="'卡牌数值'!AE$1" display="打开" xr:uid="{50FBCF09-289E-43D8-B991-6507940F89B2}"/>
+    <hyperlink ref="A65" location="'卡牌数值'!AF$1" display="打开" xr:uid="{BA40D10E-6A6D-4C71-9320-C39025038B8A}"/>
+    <hyperlink ref="A66" location="'卡牌数值'!AG$1" display="打开" xr:uid="{E7359133-6DF4-4BB5-8159-4EBEAE45F573}"/>
+    <hyperlink ref="A17" location="'卡牌数值'!AH$1" display="打开" xr:uid="{AB91E30C-A5D7-4E7A-A61D-41A3E0D35D08}"/>
+    <hyperlink ref="A70" location="'卡牌数值'!AI$1" display="打开" xr:uid="{926107FF-A01A-4B95-932D-0584C00F628A}"/>
+    <hyperlink ref="A38" location="'卡牌数值'!AJ$1" display="打开" xr:uid="{F5DBD22A-02C9-40EC-BC99-77935BA64D70}"/>
+    <hyperlink ref="A41" location="'卡牌数值'!AK$1" display="打开" xr:uid="{45592DD4-8458-41AE-A9EC-7EF169D236BD}"/>
+    <hyperlink ref="A39" location="'卡牌数值'!AL$1" display="打开" xr:uid="{727F22BB-146F-4079-A44F-B06D97D4AC09}"/>
+    <hyperlink ref="A40" location="'卡牌数值'!AM$1" display="打开" xr:uid="{951AF928-7F47-479C-AE1E-069EE9003DA2}"/>
+    <hyperlink ref="A68" location="'卡牌数值'!AN$1" display="打开" xr:uid="{DA51AC90-26DC-400D-9D14-D5F1F468B4C0}"/>
+    <hyperlink ref="A73" location="'卡牌数值'!AO$1" display="打开" xr:uid="{AB970096-ABF3-4F48-87B5-B66A9C0E2CBE}"/>
+    <hyperlink ref="A75" location="'卡牌数值'!AP$1" display="打开" xr:uid="{C8EF8F37-3AAB-456B-8D89-241296B5D9D9}"/>
+    <hyperlink ref="A72" location="'卡牌数值'!AQ$1" display="打开" xr:uid="{EE5E7272-26E1-4E03-8096-0B1593675822}"/>
+    <hyperlink ref="A71" location="'卡牌数值'!AR$1" display="打开" xr:uid="{B4E54A05-6E17-4CFD-8D18-682238136783}"/>
+    <hyperlink ref="A5" location="'卡牌数值'!AS$1" display="打开" xr:uid="{98D4FC13-1FC4-48C1-B0E2-CF7572E5D753}"/>
+    <hyperlink ref="A22" location="'卡牌数值'!AT$1" display="打开" xr:uid="{0883F911-6734-4004-9977-115BD16EA24E}"/>
+    <hyperlink ref="A23" location="'卡牌数值'!AU$1" display="打开" xr:uid="{544FF932-B903-4FA2-B2C6-F94A8EAA31F3}"/>
+    <hyperlink ref="A3" location="'卡牌数值'!AV$1" display="打开" xr:uid="{884E4BFA-69A1-4577-BEDA-F61BA2E51007}"/>
+    <hyperlink ref="A48" location="'卡牌数值'!AW$1" display="打开" xr:uid="{C8C86A84-EBD6-4C21-BC3E-6CEA23319579}"/>
+    <hyperlink ref="A53" location="'卡牌数值'!AX$1" display="打开" xr:uid="{A3A7FC62-0223-4D04-8470-F44C53AFFEF7}"/>
+    <hyperlink ref="A50" location="'卡牌数值'!AY$1" display="打开" xr:uid="{B911F6B2-ECA8-4845-A1E7-260D3B60DB8B}"/>
+    <hyperlink ref="A49" location="'卡牌数值'!AZ$1" display="打开" xr:uid="{734850AF-E3DB-4456-A2F0-09C56662670B}"/>
+    <hyperlink ref="A31" location="'卡牌数值'!BA$1" display="打开" xr:uid="{E43A6D34-A76F-404A-9AC5-404245F3D0B1}"/>
+    <hyperlink ref="A51" location="'卡牌数值'!BB$1" display="打开" xr:uid="{DBB7009C-E32C-4F9F-9815-FABFAEF1CFAE}"/>
+    <hyperlink ref="A2" location="'卡牌数值'!BC$1" display="打开" xr:uid="{4F4671B2-B564-4B02-831C-A23383DDE16B}"/>
+    <hyperlink ref="A21" location="'卡牌数值'!BD$1" display="打开" xr:uid="{92449BD4-4D9E-4E6F-959D-A6F34DF34540}"/>
+    <hyperlink ref="A20" location="'卡牌数值'!BE$1" display="打开" xr:uid="{2C377A93-071F-4BF8-9DE1-E2F0CD039118}"/>
+    <hyperlink ref="A19" location="'卡牌数值'!BF$1" display="打开" xr:uid="{A52B49A0-7965-4AB3-93AC-E9A2D950450F}"/>
+    <hyperlink ref="A54" location="'卡牌数值'!BG$1" display="打开" xr:uid="{AE45E290-568A-4F69-8C78-F9D7C0AE1823}"/>
+    <hyperlink ref="A43" location="'卡牌数值'!BH$1" display="打开" xr:uid="{BA91948E-BAEE-4156-BDD8-086C934B7277}"/>
+    <hyperlink ref="A45" location="'卡牌数值'!BI$1" display="打开" xr:uid="{61527EF7-98E9-438F-92F6-C69BE985E2CC}"/>
+    <hyperlink ref="A44" location="'卡牌数值'!BJ$1" display="打开" xr:uid="{D98E6492-E974-4797-A3C1-A653A44D7E2A}"/>
+    <hyperlink ref="A46" location="'卡牌数值'!BK$1" display="打开" xr:uid="{F1F00C3A-BE13-484F-A76E-0B3BA8B0C3FC}"/>
+    <hyperlink ref="A52" location="'卡牌数值'!BL$1" display="打开" xr:uid="{B0ED6633-A18C-4169-A6A1-9A7EBB7FE0D3}"/>
+    <hyperlink ref="A47" location="'卡牌数值'!BM$1" display="打开" xr:uid="{609732F7-D2CC-4A24-A626-FD641ACC6D6D}"/>
+    <hyperlink ref="A4" location="'卡牌数值'!BN$1" display="打开" xr:uid="{EFEF80F1-86D8-478D-84BB-1288F62A68B0}"/>
+    <hyperlink ref="A15" location="'卡牌数值'!BO$1" display="打开" xr:uid="{1C6FED27-915E-478E-9643-DD9488516FBE}"/>
+    <hyperlink ref="A14" location="'卡牌数值'!BP$1" display="打开" xr:uid="{5FFBEC32-02F0-4956-B1BC-1567D87129C6}"/>
+    <hyperlink ref="A33" location="'卡牌数值'!BQ$1" display="打开" xr:uid="{104350DA-59F4-4392-AC6D-79471FA9214D}"/>
+    <hyperlink ref="A35" location="'卡牌数值'!BR$1" display="打开" xr:uid="{B8E57C5C-3DFD-4592-8E4C-448C0E49C46E}"/>
+    <hyperlink ref="A56" location="'卡牌数值'!BS$1" display="打开" xr:uid="{B88F6C0B-B0A0-4525-B883-CA55AA43D751}"/>
+    <hyperlink ref="A13" location="'卡牌数值'!BT$1" display="打开" xr:uid="{C8279948-F421-443A-99CD-90A92AAF15EC}"/>
+    <hyperlink ref="A30" location="'卡牌数值'!BU$1" display="打开" xr:uid="{9892057E-6828-4E38-BA76-A9427AE8F6BB}"/>
+    <hyperlink ref="A42" location="'卡牌数值'!BV$1" display="打开" xr:uid="{01E371DC-B222-4E6D-BA1E-6454C2AFD7E5}"/>
+    <hyperlink ref="A18" location="'卡牌数值'!BW$1" display="打开" xr:uid="{DFF53BFC-5C03-4ED0-81C2-97F1ADED3A59}"/>
+    <hyperlink ref="A74" location="'卡牌数值'!BX$1" display="打开" xr:uid="{847C8C97-F6A2-44EA-92F9-83891ED67DF3}"/>
+    <hyperlink ref="A69" location="'卡牌数值'!BY$1" display="打开" xr:uid="{52A61958-7E12-474B-8FF4-A98C6BC4E35A}"/>
+    <hyperlink ref="A64" location="'卡牌数值'!BZ$1" display="打开" xr:uid="{2433F839-C576-4850-A4A6-88C4EBBAE338}"/>
+    <hyperlink ref="A16" location="'卡牌数值'!CA$1" display="打开" xr:uid="{B3CFF3A1-6F76-4D90-A0AB-5D86882A2971}"/>
+    <hyperlink ref="A29" location="'卡牌数值'!CB$1" display="打开" xr:uid="{C348F711-1400-434A-9E65-B9768DC1B735}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F953D376-2557-4FFE-A3D2-588E7C73D0D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72001FFE-9B33-4D7C-A446-13BC21F96CC7}">
   <dimension ref="A1:CB89"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -6342,7 +6342,7 @@
         <v>30</v>
       </c>
       <c r="AK4" s="11" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="AL4" s="11" t="s">
         <v>30</v>
@@ -8008,7 +8008,7 @@
         <v>30</v>
       </c>
       <c r="AK11" s="14" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="AL11" s="14" t="s">
         <v>30</v>
@@ -9908,7 +9908,9 @@
       </c>
       <c r="D22" s="15"/>
       <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
+      <c r="F22" s="15">
+        <v>15</v>
+      </c>
       <c r="G22" s="15"/>
       <c r="H22" s="15"/>
       <c r="I22" s="15"/>
@@ -14280,7 +14282,9 @@
       <c r="BO69" s="15"/>
       <c r="BP69" s="15"/>
       <c r="BQ69" s="15"/>
-      <c r="BR69" s="15"/>
+      <c r="BR69" s="15">
+        <v>3</v>
+      </c>
       <c r="BS69" s="15"/>
       <c r="BT69" s="15"/>
       <c r="BU69" s="15"/>
@@ -15038,7 +15042,7 @@
       <c r="CA77" s="15"/>
       <c r="CB77" s="15"/>
     </row>
-    <row r="78" spans="1:80" ht="58" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:80" ht="72.5" x14ac:dyDescent="0.3">
       <c r="A78" s="12" t="s">
         <v>561</v>
       </c>
@@ -16721,7 +16725,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E28E3187-D08D-4CF7-8F0F-F2A2D1213499}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A8C27C0-327A-4BD6-AF82-3A6BF51D7516}">
   <dimension ref="A1:D85"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -17911,7 +17915,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D99EF2DB-C638-45E5-924F-240A85917DD7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FDAE2B4-2075-44CD-BE6D-8EC119551F35}">
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>